<commit_message>
Convert FIRE planner to Indian Rupees (₹ INR)
- Replace all $ currency symbols with ₹ throughout
- Default values now reflect Indian financial context:
  · Portfolio: ₹20L starting, ₹50K/month SIP
  · Income: ₹1L primary salary, ₹60K spouse
  · Assets: EPF, PPF, NPS, Equity MF, SGB, FD
  · Liabilities: Home Loan @ 8.5%, Car Loan, Education Loan
  · Expenses: Indian categories (Zomato, Ola, Kirana, EMI)
  · Savings: VPF, PPF, NPS Tier-1, SIP, Direct Stocks
- Rates updated for India: 12% equity return, 6% CPI inflation
- SWR notes updated with India-specific context
- Added India flag and INR labels to sheet headers

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015X4vvhhjNcsxK1mvBr2kB8
</commit_message>
<xml_diff>
--- a/FIRE_Retirement_Planner.xlsx
+++ b/FIRE_Retirement_Planner.xlsx
@@ -21,10 +21,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="6">
-    <numFmt numFmtId="164" formatCode="$#,##0"/>
+    <numFmt numFmtId="164" formatCode="₹#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
-    <numFmt numFmtId="167" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="₹#,##0.00"/>
     <numFmt numFmtId="168" formatCode="0.0&quot;%&quot;"/>
     <numFmt numFmtId="169" formatCode="0.0 &quot;yrs&quot;"/>
   </numFmts>
@@ -285,7 +285,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="15"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -1550,14 +1550,14 @@
     <row r="2" ht="48" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>FIRE RETIREMENT PLANNER</t>
+          <t>FIRE RETIREMENT PLANNER  🇮🇳</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Financial Independence · Retire Early · Live Free</t>
+          <t>Financial Independence · Retire Early · Live Free  ·  All values in ₹ Indian Rupees (INR)</t>
         </is>
       </c>
     </row>
@@ -1913,14 +1913,14 @@
     <row r="2" ht="44" customHeight="1">
       <c r="B2" s="23" t="inlineStr">
         <is>
-          <t>NET WORTH TRACKER</t>
+          <t>NET WORTH TRACKER  (₹ Indian Rupees)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="24" t="inlineStr">
         <is>
-          <t>Last updated: June 24, 2026  ·  Update monthly for accurate FIRE tracking</t>
+          <t>Last updated: June 25, 2026  ·  Update monthly for accurate FIRE tracking  ·  Amounts in ₹ INR</t>
         </is>
       </c>
     </row>
@@ -1962,144 +1962,144 @@
     <row r="7" ht="18" customHeight="1">
       <c r="B7" s="26" t="inlineStr">
         <is>
-          <t>Cash &amp; Savings Account</t>
+          <t>Savings Bank Account</t>
         </is>
       </c>
       <c r="C7" s="27" t="n">
-        <v>15000</v>
+        <v>500000</v>
       </c>
       <c r="D7" s="28">
         <f>IF(C21&gt;0,C7/C21,0)</f>
         <v/>
       </c>
       <c r="E7" s="29" t="n">
-        <v>0.005</v>
+        <v>0.035</v>
       </c>
       <c r="F7" s="30" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="26" t="inlineStr">
         <is>
-          <t>Emergency Fund</t>
+          <t>Emergency Fund (FD / Liquid MF)</t>
         </is>
       </c>
       <c r="C8" s="27" t="n">
-        <v>10000</v>
+        <v>300000</v>
       </c>
       <c r="D8" s="28">
         <f>IF(C21&gt;0,C8/C21,0)</f>
         <v/>
       </c>
       <c r="E8" s="29" t="n">
-        <v>0.047</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="F8" s="30" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="26" t="inlineStr">
         <is>
-          <t>Checking Account</t>
+          <t>Salary / Current Account</t>
         </is>
       </c>
       <c r="C9" s="27" t="n">
-        <v>5000</v>
+        <v>100000</v>
       </c>
       <c r="D9" s="28">
         <f>IF(C21&gt;0,C9/C21,0)</f>
         <v/>
       </c>
       <c r="E9" s="29" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="F9" s="30" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="B10" s="26" t="inlineStr">
         <is>
-          <t>401(k) / 403(b)</t>
+          <t>EPF (Employee Provident Fund)</t>
         </is>
       </c>
       <c r="C10" s="27" t="n">
-        <v>85000</v>
+        <v>2000000</v>
       </c>
       <c r="D10" s="28">
         <f>IF(C21&gt;0,C10/C21,0)</f>
         <v/>
       </c>
       <c r="E10" s="29" t="n">
-        <v>0.08</v>
+        <v>0.082</v>
       </c>
       <c r="F10" s="30" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="B11" s="26" t="inlineStr">
         <is>
-          <t>Roth IRA</t>
+          <t>PPF (Public Provident Fund)</t>
         </is>
       </c>
       <c r="C11" s="27" t="n">
-        <v>35000</v>
+        <v>800000</v>
       </c>
       <c r="D11" s="28">
         <f>IF(C21&gt;0,C11/C21,0)</f>
         <v/>
       </c>
       <c r="E11" s="29" t="n">
-        <v>0.08</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="F11" s="30" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="26" t="inlineStr">
         <is>
-          <t>Traditional IRA</t>
+          <t>NPS (National Pension System)</t>
         </is>
       </c>
       <c r="C12" s="27" t="n">
-        <v>0</v>
+        <v>500000</v>
       </c>
       <c r="D12" s="28">
         <f>IF(C21&gt;0,C12/C21,0)</f>
         <v/>
       </c>
       <c r="E12" s="29" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="F12" s="30" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="B13" s="26" t="inlineStr">
         <is>
-          <t>Taxable Brokerage Account</t>
+          <t>Mutual Funds — Equity (Demat)</t>
         </is>
       </c>
       <c r="C13" s="27" t="n">
-        <v>25000</v>
+        <v>1200000</v>
       </c>
       <c r="D13" s="28">
         <f>IF(C21&gt;0,C13/C21,0)</f>
         <v/>
       </c>
       <c r="E13" s="29" t="n">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
       <c r="F13" s="30" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="B14" s="26" t="inlineStr">
         <is>
-          <t>HSA (Health Savings Account)</t>
+          <t>Stocks — Direct Equity</t>
         </is>
       </c>
       <c r="C14" s="27" t="n">
-        <v>8000</v>
+        <v>600000</v>
       </c>
       <c r="D14" s="28">
         <f>IF(C21&gt;0,C14/C21,0)</f>
         <v/>
       </c>
       <c r="E14" s="29" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.12</v>
       </c>
       <c r="F14" s="30" t="n"/>
     </row>
@@ -2110,14 +2110,14 @@
         </is>
       </c>
       <c r="C15" s="27" t="n">
-        <v>350000</v>
+        <v>8000000</v>
       </c>
       <c r="D15" s="28">
         <f>IF(C21&gt;0,C15/C21,0)</f>
         <v/>
       </c>
       <c r="E15" s="29" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="F15" s="30" t="n"/>
     </row>
@@ -2135,43 +2135,43 @@
         <v/>
       </c>
       <c r="E16" s="29" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="F16" s="30" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="26" t="inlineStr">
         <is>
-          <t>Vehicles</t>
+          <t>Gold / Sovereign Gold Bonds</t>
         </is>
       </c>
       <c r="C17" s="27" t="n">
-        <v>15000</v>
+        <v>500000</v>
       </c>
       <c r="D17" s="28">
         <f>IF(C21&gt;0,C17/C21,0)</f>
         <v/>
       </c>
-      <c r="E17" s="31" t="n">
-        <v>-0.1</v>
+      <c r="E17" s="29" t="n">
+        <v>0.08</v>
       </c>
       <c r="F17" s="30" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="26" t="inlineStr">
         <is>
-          <t>Business Equity</t>
+          <t>Vehicles</t>
         </is>
       </c>
       <c r="C18" s="27" t="n">
-        <v>0</v>
+        <v>600000</v>
       </c>
       <c r="D18" s="28">
         <f>IF(C21&gt;0,C18/C21,0)</f>
         <v/>
       </c>
-      <c r="E18" s="29" t="n">
-        <v>0.1</v>
+      <c r="E18" s="31" t="n">
+        <v>-0.15</v>
       </c>
       <c r="F18" s="30" t="n"/>
     </row>
@@ -2182,7 +2182,7 @@
         </is>
       </c>
       <c r="C19" s="27" t="n">
-        <v>5000</v>
+        <v>200000</v>
       </c>
       <c r="D19" s="28">
         <f>IF(C21&gt;0,C19/C21,0)</f>
@@ -2200,14 +2200,14 @@
         </is>
       </c>
       <c r="C20" s="27" t="n">
-        <v>2000</v>
+        <v>100000</v>
       </c>
       <c r="D20" s="28">
         <f>IF(C21&gt;0,C20/C21,0)</f>
         <v/>
       </c>
       <c r="E20" s="29" t="n">
-        <v>0.02</v>
+        <v>0.05</v>
       </c>
       <c r="F20" s="30" t="n"/>
     </row>
@@ -2269,25 +2269,25 @@
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="26" t="inlineStr">
         <is>
-          <t>Mortgage — Primary Residence</t>
+          <t>Home Loan — Primary Residence</t>
         </is>
       </c>
       <c r="C25" s="27" t="n">
-        <v>250000</v>
+        <v>4000000</v>
       </c>
       <c r="D25" s="31">
         <f>IF(C37&gt;0,C25/C37,0)</f>
         <v/>
       </c>
       <c r="E25" s="36" t="n">
-        <v>0.065</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="F25" s="37" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="B26" s="26" t="inlineStr">
         <is>
-          <t>Mortgage — Investment Property</t>
+          <t>Home Loan — Investment Property</t>
         </is>
       </c>
       <c r="C26" s="27" t="n">
@@ -2298,14 +2298,14 @@
         <v/>
       </c>
       <c r="E26" s="36" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.09</v>
       </c>
       <c r="F26" s="37" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="B27" s="26" t="inlineStr">
         <is>
-          <t>Home Equity Loan / HELOC</t>
+          <t>Loan Against Property (LAP)</t>
         </is>
       </c>
       <c r="C27" s="27" t="n">
@@ -2315,33 +2315,33 @@
         <f>IF(C37&gt;0,C27/C37,0)</f>
         <v/>
       </c>
-      <c r="E27" s="36" t="n">
-        <v>0.08500000000000001</v>
+      <c r="E27" s="31" t="n">
+        <v>0.105</v>
       </c>
       <c r="F27" s="37" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="B28" s="26" t="inlineStr">
         <is>
-          <t>Auto Loan 1</t>
+          <t>Car Loan 1</t>
         </is>
       </c>
       <c r="C28" s="27" t="n">
-        <v>12000</v>
+        <v>600000</v>
       </c>
       <c r="D28" s="31">
         <f>IF(C37&gt;0,C28/C37,0)</f>
         <v/>
       </c>
       <c r="E28" s="36" t="n">
-        <v>0.059</v>
+        <v>0.09</v>
       </c>
       <c r="F28" s="37" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="B29" s="26" t="inlineStr">
         <is>
-          <t>Auto Loan 2</t>
+          <t>Car Loan 2</t>
         </is>
       </c>
       <c r="C29" s="27" t="n">
@@ -2359,18 +2359,18 @@
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="26" t="inlineStr">
         <is>
-          <t>Student Loans</t>
+          <t>Education Loan</t>
         </is>
       </c>
       <c r="C30" s="27" t="n">
-        <v>18000</v>
+        <v>500000</v>
       </c>
       <c r="D30" s="31">
         <f>IF(C37&gt;0,C30/C37,0)</f>
         <v/>
       </c>
       <c r="E30" s="36" t="n">
-        <v>0.055</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="F30" s="37" t="n"/>
     </row>
@@ -2381,14 +2381,14 @@
         </is>
       </c>
       <c r="C31" s="27" t="n">
-        <v>3500</v>
+        <v>100000</v>
       </c>
       <c r="D31" s="31">
         <f>IF(C37&gt;0,C31/C37,0)</f>
         <v/>
       </c>
       <c r="E31" s="31" t="n">
-        <v>0.22</v>
+        <v>0.36</v>
       </c>
       <c r="F31" s="37" t="n"/>
     </row>
@@ -2406,7 +2406,7 @@
         <v/>
       </c>
       <c r="E32" s="31" t="n">
-        <v>0.22</v>
+        <v>0.36</v>
       </c>
       <c r="F32" s="37" t="n"/>
     </row>
@@ -2424,14 +2424,14 @@
         <v/>
       </c>
       <c r="E33" s="31" t="n">
-        <v>0.12</v>
+        <v>0.14</v>
       </c>
       <c r="F33" s="37" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="26" t="inlineStr">
         <is>
-          <t>Medical Debt</t>
+          <t>Medical / Emergency Loan</t>
         </is>
       </c>
       <c r="C34" s="27" t="n">
@@ -2449,7 +2449,7 @@
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="26" t="inlineStr">
         <is>
-          <t>Business Debt</t>
+          <t>Business Loan</t>
         </is>
       </c>
       <c r="C35" s="27" t="n">
@@ -2459,8 +2459,8 @@
         <f>IF(C37&gt;0,C35/C37,0)</f>
         <v/>
       </c>
-      <c r="E35" s="36" t="n">
-        <v>0.08</v>
+      <c r="E35" s="31" t="n">
+        <v>0.12</v>
       </c>
       <c r="F35" s="37" t="n"/>
     </row>
@@ -2640,14 +2640,14 @@
     <row r="2" ht="44" customHeight="1">
       <c r="B2" s="23" t="inlineStr">
         <is>
-          <t>MONTHLY BUDGET &amp; SAVINGS RATE</t>
+          <t>MONTHLY BUDGET &amp; SAVINGS RATE  (₹ INR)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="24" t="inlineStr">
         <is>
-          <t>Savings Rate is the single most important variable for achieving FIRE</t>
+          <t>Savings Rate is the single most important variable for achieving FIRE  ·  All amounts in ₹ INR</t>
         </is>
       </c>
     </row>
@@ -2694,14 +2694,14 @@
     <row r="7" ht="18" customHeight="1">
       <c r="B7" s="26" t="inlineStr">
         <is>
-          <t>Primary Job — Net Take-Home Pay</t>
+          <t>Primary Salary — Net In-Hand (after TDS)</t>
         </is>
       </c>
       <c r="C7" s="27" t="n">
-        <v>6500</v>
+        <v>100000</v>
       </c>
       <c r="D7" s="27" t="n">
-        <v>6500</v>
+        <v>100000</v>
       </c>
       <c r="E7" s="59">
         <f>D7-C7</f>
@@ -2719,14 +2719,14 @@
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="26" t="inlineStr">
         <is>
-          <t>Spouse / Partner Income</t>
+          <t>Spouse / Partner In-Hand Salary</t>
         </is>
       </c>
       <c r="C8" s="27" t="n">
-        <v>4000</v>
+        <v>60000</v>
       </c>
       <c r="D8" s="27" t="n">
-        <v>4000</v>
+        <v>60000</v>
       </c>
       <c r="E8" s="59">
         <f>D8-C8</f>
@@ -2744,14 +2744,14 @@
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="26" t="inlineStr">
         <is>
-          <t>Side Hustle / Freelance</t>
+          <t>Freelance / Consulting Income</t>
         </is>
       </c>
       <c r="C9" s="27" t="n">
-        <v>500</v>
+        <v>10000</v>
       </c>
       <c r="D9" s="27" t="n">
-        <v>500</v>
+        <v>10000</v>
       </c>
       <c r="E9" s="59">
         <f>D9-C9</f>
@@ -2798,10 +2798,10 @@
         </is>
       </c>
       <c r="C11" s="27" t="n">
-        <v>200</v>
+        <v>5000</v>
       </c>
       <c r="D11" s="27" t="n">
-        <v>200</v>
+        <v>5000</v>
       </c>
       <c r="E11" s="59">
         <f>D11-C11</f>
@@ -2880,14 +2880,14 @@
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="26" t="inlineStr">
         <is>
-          <t>Rent / Mortgage Payment</t>
+          <t>Rent / Home Loan EMI</t>
         </is>
       </c>
       <c r="C16" s="27" t="n">
-        <v>2200</v>
+        <v>30000</v>
       </c>
       <c r="D16" s="27" t="n">
-        <v>2200</v>
+        <v>30000</v>
       </c>
       <c r="E16" s="59">
         <f>D16-C16</f>
@@ -2905,14 +2905,14 @@
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="26" t="inlineStr">
         <is>
-          <t>HOA Fees</t>
+          <t>Society Maintenance Charges</t>
         </is>
       </c>
       <c r="C17" s="27" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="D17" s="27" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="E17" s="59">
         <f>D17-C17</f>
@@ -2930,14 +2930,14 @@
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="26" t="inlineStr">
         <is>
-          <t>Homeowner's / Renter's Insurance</t>
+          <t>Home / Renter's Insurance</t>
         </is>
       </c>
       <c r="C18" s="27" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="D18" s="27" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E18" s="59">
         <f>D18-C18</f>
@@ -2955,14 +2955,14 @@
     <row r="19" ht="18" customHeight="1">
       <c r="B19" s="26" t="inlineStr">
         <is>
-          <t>Car Payment 1</t>
+          <t>Car Loan EMI 1</t>
         </is>
       </c>
       <c r="C19" s="27" t="n">
-        <v>350</v>
+        <v>8000</v>
       </c>
       <c r="D19" s="27" t="n">
-        <v>350</v>
+        <v>8000</v>
       </c>
       <c r="E19" s="59">
         <f>D19-C19</f>
@@ -2980,7 +2980,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="B20" s="26" t="inlineStr">
         <is>
-          <t>Car Payment 2</t>
+          <t>Car Loan EMI 2</t>
         </is>
       </c>
       <c r="C20" s="27" t="n">
@@ -3005,14 +3005,14 @@
     <row r="21" ht="18" customHeight="1">
       <c r="B21" s="26" t="inlineStr">
         <is>
-          <t>Auto Insurance</t>
+          <t>Vehicle Insurance</t>
         </is>
       </c>
       <c r="C21" s="27" t="n">
-        <v>150</v>
+        <v>3000</v>
       </c>
       <c r="D21" s="27" t="n">
-        <v>150</v>
+        <v>3000</v>
       </c>
       <c r="E21" s="59">
         <f>D21-C21</f>
@@ -3034,10 +3034,10 @@
         </is>
       </c>
       <c r="C22" s="27" t="n">
-        <v>400</v>
+        <v>5000</v>
       </c>
       <c r="D22" s="27" t="n">
-        <v>400</v>
+        <v>5000</v>
       </c>
       <c r="E22" s="59">
         <f>D22-C22</f>
@@ -3055,14 +3055,14 @@
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="26" t="inlineStr">
         <is>
-          <t>Life / Disability Insurance</t>
+          <t>Term Life Insurance Premium</t>
         </is>
       </c>
       <c r="C23" s="27" t="n">
-        <v>50</v>
+        <v>2500</v>
       </c>
       <c r="D23" s="27" t="n">
-        <v>50</v>
+        <v>2500</v>
       </c>
       <c r="E23" s="59">
         <f>D23-C23</f>
@@ -3080,14 +3080,14 @@
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="26" t="inlineStr">
         <is>
-          <t>Internet</t>
+          <t>Internet (Broadband + Mobile)</t>
         </is>
       </c>
       <c r="C24" s="27" t="n">
-        <v>80</v>
+        <v>1500</v>
       </c>
       <c r="D24" s="27" t="n">
-        <v>80</v>
+        <v>1500</v>
       </c>
       <c r="E24" s="59">
         <f>D24-C24</f>
@@ -3105,14 +3105,14 @@
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="26" t="inlineStr">
         <is>
-          <t>Phone</t>
+          <t>Mobile / DTH Recharge</t>
         </is>
       </c>
       <c r="C25" s="27" t="n">
-        <v>85</v>
+        <v>1000</v>
       </c>
       <c r="D25" s="27" t="n">
-        <v>85</v>
+        <v>1000</v>
       </c>
       <c r="E25" s="59">
         <f>D25-C25</f>
@@ -3130,14 +3130,14 @@
     <row r="26" ht="18" customHeight="1">
       <c r="B26" s="26" t="inlineStr">
         <is>
-          <t>Streaming Subscriptions</t>
+          <t>OTT Subscriptions (Netflix etc.)</t>
         </is>
       </c>
       <c r="C26" s="27" t="n">
-        <v>50</v>
+        <v>1000</v>
       </c>
       <c r="D26" s="27" t="n">
-        <v>50</v>
+        <v>1000</v>
       </c>
       <c r="E26" s="59">
         <f>D26-C26</f>
@@ -3159,10 +3159,10 @@
         </is>
       </c>
       <c r="C27" s="27" t="n">
-        <v>40</v>
+        <v>1500</v>
       </c>
       <c r="D27" s="27" t="n">
-        <v>40</v>
+        <v>1500</v>
       </c>
       <c r="E27" s="59">
         <f>D27-C27</f>
@@ -3215,14 +3215,14 @@
     <row r="31" ht="18" customHeight="1">
       <c r="B31" s="26" t="inlineStr">
         <is>
-          <t>Groceries &amp; Household Supplies</t>
+          <t>Groceries &amp; Kirana / Supermarket</t>
         </is>
       </c>
       <c r="C31" s="27" t="n">
-        <v>600</v>
+        <v>12000</v>
       </c>
       <c r="D31" s="27" t="n">
-        <v>600</v>
+        <v>12000</v>
       </c>
       <c r="E31" s="59">
         <f>D31-C31</f>
@@ -3240,14 +3240,14 @@
     <row r="32" ht="18" customHeight="1">
       <c r="B32" s="26" t="inlineStr">
         <is>
-          <t>Dining Out &amp; Takeout</t>
+          <t>Dining Out, Zomato &amp; Swiggy</t>
         </is>
       </c>
       <c r="C32" s="27" t="n">
-        <v>200</v>
+        <v>5000</v>
       </c>
       <c r="D32" s="27" t="n">
-        <v>200</v>
+        <v>5000</v>
       </c>
       <c r="E32" s="59">
         <f>D32-C32</f>
@@ -3265,14 +3265,14 @@
     <row r="33" ht="18" customHeight="1">
       <c r="B33" s="26" t="inlineStr">
         <is>
-          <t>Gas &amp; Transportation</t>
+          <t>Petrol / CNG &amp; Transport</t>
         </is>
       </c>
       <c r="C33" s="27" t="n">
-        <v>150</v>
+        <v>5000</v>
       </c>
       <c r="D33" s="27" t="n">
-        <v>150</v>
+        <v>5000</v>
       </c>
       <c r="E33" s="59">
         <f>D33-C33</f>
@@ -3290,14 +3290,14 @@
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="26" t="inlineStr">
         <is>
-          <t>Parking, Tolls &amp; Rideshare</t>
+          <t>Auto, Cab (Ola/Uber) &amp; Parking</t>
         </is>
       </c>
       <c r="C34" s="27" t="n">
-        <v>30</v>
+        <v>2000</v>
       </c>
       <c r="D34" s="27" t="n">
-        <v>30</v>
+        <v>2000</v>
       </c>
       <c r="E34" s="59">
         <f>D34-C34</f>
@@ -3315,14 +3315,14 @@
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="26" t="inlineStr">
         <is>
-          <t>Clothing &amp; Apparel</t>
+          <t>Clothing &amp; Lifestyle Shopping</t>
         </is>
       </c>
       <c r="C35" s="27" t="n">
-        <v>100</v>
+        <v>5000</v>
       </c>
       <c r="D35" s="27" t="n">
-        <v>100</v>
+        <v>5000</v>
       </c>
       <c r="E35" s="59">
         <f>D35-C35</f>
@@ -3340,14 +3340,14 @@
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="26" t="inlineStr">
         <is>
-          <t>Entertainment &amp; Recreation</t>
+          <t>Entertainment &amp; Movies / Events</t>
         </is>
       </c>
       <c r="C36" s="27" t="n">
-        <v>100</v>
+        <v>3000</v>
       </c>
       <c r="D36" s="27" t="n">
-        <v>100</v>
+        <v>3000</v>
       </c>
       <c r="E36" s="59">
         <f>D36-C36</f>
@@ -3365,14 +3365,14 @@
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="26" t="inlineStr">
         <is>
-          <t>Travel &amp; Vacation</t>
+          <t>Travel &amp; Holidays</t>
         </is>
       </c>
       <c r="C37" s="27" t="n">
-        <v>200</v>
+        <v>8000</v>
       </c>
       <c r="D37" s="27" t="n">
-        <v>200</v>
+        <v>8000</v>
       </c>
       <c r="E37" s="59">
         <f>D37-C37</f>
@@ -3390,14 +3390,14 @@
     <row r="38" ht="18" customHeight="1">
       <c r="B38" s="26" t="inlineStr">
         <is>
-          <t>Personal Care &amp; Beauty</t>
+          <t>Personal Care &amp; Salon</t>
         </is>
       </c>
       <c r="C38" s="27" t="n">
-        <v>80</v>
+        <v>2000</v>
       </c>
       <c r="D38" s="27" t="n">
-        <v>80</v>
+        <v>2000</v>
       </c>
       <c r="E38" s="59">
         <f>D38-C38</f>
@@ -3415,14 +3415,14 @@
     <row r="39" ht="18" customHeight="1">
       <c r="B39" s="26" t="inlineStr">
         <is>
-          <t>Medical, Dental &amp; Pharmacy</t>
+          <t>Medical, Doctor &amp; Pharmacy</t>
         </is>
       </c>
       <c r="C39" s="27" t="n">
-        <v>50</v>
+        <v>3000</v>
       </c>
       <c r="D39" s="27" t="n">
-        <v>50</v>
+        <v>3000</v>
       </c>
       <c r="E39" s="59">
         <f>D39-C39</f>
@@ -3444,10 +3444,10 @@
         </is>
       </c>
       <c r="C40" s="27" t="n">
-        <v>100</v>
+        <v>2000</v>
       </c>
       <c r="D40" s="27" t="n">
-        <v>100</v>
+        <v>2000</v>
       </c>
       <c r="E40" s="59">
         <f>D40-C40</f>
@@ -3465,14 +3465,14 @@
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="26" t="inlineStr">
         <is>
-          <t>Gifts &amp; Charitable Donations</t>
+          <t>Gifts, Pooja &amp; Charitable Donations</t>
         </is>
       </c>
       <c r="C41" s="27" t="n">
-        <v>75</v>
+        <v>3000</v>
       </c>
       <c r="D41" s="27" t="n">
-        <v>75</v>
+        <v>3000</v>
       </c>
       <c r="E41" s="59">
         <f>D41-C41</f>
@@ -3515,7 +3515,7 @@
     <row r="43" ht="18" customHeight="1">
       <c r="B43" s="26" t="inlineStr">
         <is>
-          <t>Childcare &amp; Education</t>
+          <t>Children's School Fees &amp; Tuition</t>
         </is>
       </c>
       <c r="C43" s="27" t="n">
@@ -3540,14 +3540,14 @@
     <row r="44" ht="18" customHeight="1">
       <c r="B44" s="26" t="inlineStr">
         <is>
-          <t>Miscellaneous / Catch-All</t>
+          <t>Miscellaneous / Unplanned</t>
         </is>
       </c>
       <c r="C44" s="27" t="n">
-        <v>100</v>
+        <v>3000</v>
       </c>
       <c r="D44" s="27" t="n">
-        <v>100</v>
+        <v>3000</v>
       </c>
       <c r="E44" s="59">
         <f>D44-C44</f>
@@ -3600,14 +3600,14 @@
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="26" t="inlineStr">
         <is>
-          <t>401(k) / 403(b) Contribution</t>
+          <t>EPF Voluntary Contribution (VPF)</t>
         </is>
       </c>
       <c r="C48" s="27" t="n">
-        <v>1000</v>
+        <v>5000</v>
       </c>
       <c r="D48" s="27" t="n">
-        <v>1000</v>
+        <v>5000</v>
       </c>
       <c r="E48" s="59">
         <f>D48-C48</f>
@@ -3625,14 +3625,14 @@
     <row r="49" ht="18" customHeight="1">
       <c r="B49" s="26" t="inlineStr">
         <is>
-          <t>Roth IRA Contribution</t>
+          <t>PPF Contribution</t>
         </is>
       </c>
       <c r="C49" s="27" t="n">
-        <v>500</v>
+        <v>5000</v>
       </c>
       <c r="D49" s="27" t="n">
-        <v>500</v>
+        <v>5000</v>
       </c>
       <c r="E49" s="59">
         <f>D49-C49</f>
@@ -3650,14 +3650,14 @@
     <row r="50" ht="18" customHeight="1">
       <c r="B50" s="26" t="inlineStr">
         <is>
-          <t>HSA Contribution</t>
+          <t>NPS Tier-1 / Tier-2 Contribution</t>
         </is>
       </c>
       <c r="C50" s="27" t="n">
-        <v>300</v>
+        <v>5000</v>
       </c>
       <c r="D50" s="27" t="n">
-        <v>300</v>
+        <v>5000</v>
       </c>
       <c r="E50" s="59">
         <f>D50-C50</f>
@@ -3675,14 +3675,14 @@
     <row r="51" ht="18" customHeight="1">
       <c r="B51" s="26" t="inlineStr">
         <is>
-          <t>Taxable Brokerage Investment</t>
+          <t>Mutual Funds SIP — Equity</t>
         </is>
       </c>
       <c r="C51" s="27" t="n">
-        <v>500</v>
+        <v>20000</v>
       </c>
       <c r="D51" s="27" t="n">
-        <v>500</v>
+        <v>20000</v>
       </c>
       <c r="E51" s="59">
         <f>D51-C51</f>
@@ -3700,14 +3700,14 @@
     <row r="52" ht="18" customHeight="1">
       <c r="B52" s="26" t="inlineStr">
         <is>
-          <t>Emergency Fund Top-Up</t>
+          <t>Direct Stocks / ETF Investment</t>
         </is>
       </c>
       <c r="C52" s="27" t="n">
-        <v>200</v>
+        <v>10000</v>
       </c>
       <c r="D52" s="27" t="n">
-        <v>200</v>
+        <v>10000</v>
       </c>
       <c r="E52" s="59">
         <f>D52-C52</f>
@@ -3725,14 +3725,14 @@
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="26" t="inlineStr">
         <is>
-          <t>House / Goal Savings Fund</t>
+          <t>Emergency Fund / Liquid FD Top-Up</t>
         </is>
       </c>
       <c r="C53" s="27" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="D53" s="27" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="E53" s="59">
         <f>D53-C53</f>
@@ -3750,7 +3750,7 @@
     <row r="54" ht="18" customHeight="1">
       <c r="B54" s="26" t="inlineStr">
         <is>
-          <t>Other Savings / Sinking Funds</t>
+          <t>Goal-based Savings (Travel, Car)</t>
         </is>
       </c>
       <c r="C54" s="27" t="n">
@@ -3991,7 +3991,7 @@
     <row r="2" ht="44" customHeight="1">
       <c r="B2" s="23" t="inlineStr">
         <is>
-          <t>INVESTMENT GROWTH PROJECTIONS</t>
+          <t>INVESTMENT GROWTH PROJECTIONS  (₹ INR)</t>
         </is>
       </c>
     </row>
@@ -4031,7 +4031,7 @@
       </c>
       <c r="F6" s="99" t="inlineStr">
         <is>
-          <t>Lean FIRE  (20× expenses)</t>
+          <t>Lean FIRE  (20× expenses — frugal)</t>
         </is>
       </c>
       <c r="G6" s="100">
@@ -4042,11 +4042,11 @@
     <row r="7" ht="22" customHeight="1">
       <c r="B7" s="96" t="inlineStr">
         <is>
-          <t>Annual Return Rate (nominal)</t>
+          <t>Annual Return Rate — Indian Equity</t>
         </is>
       </c>
       <c r="C7" s="101" t="n">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
       <c r="D7" s="98" t="inlineStr">
         <is>
@@ -4066,11 +4066,11 @@
     <row r="8" ht="22" customHeight="1">
       <c r="B8" s="96" t="inlineStr">
         <is>
-          <t>Inflation Rate</t>
+          <t>Inflation Rate (India CPI average)</t>
         </is>
       </c>
       <c r="C8" s="101" t="n">
-        <v>0.03</v>
+        <v>0.06</v>
       </c>
       <c r="D8" s="98" t="inlineStr">
         <is>
@@ -4079,7 +4079,7 @@
       </c>
       <c r="F8" s="99" t="inlineStr">
         <is>
-          <t>Fat FIRE  (33× expenses)</t>
+          <t>Fat FIRE  (33× expenses — comfortable)</t>
         </is>
       </c>
       <c r="G8" s="100">
@@ -4090,7 +4090,7 @@
     <row r="9" ht="22" customHeight="1">
       <c r="B9" s="96" t="inlineStr">
         <is>
-          <t>Real Return Rate (nom - inflation)</t>
+          <t>Real Return Rate (nominal - inflation)</t>
         </is>
       </c>
       <c r="C9" s="102">
@@ -4104,7 +4104,7 @@
       </c>
       <c r="F9" s="99" t="inlineStr">
         <is>
-          <t>Barista FIRE  (15× expenses)</t>
+          <t>CoastFIRE  (15× expenses)</t>
         </is>
       </c>
       <c r="G9" s="100">
@@ -4115,11 +4115,11 @@
     <row r="10" ht="22" customHeight="1">
       <c r="B10" s="96" t="inlineStr">
         <is>
-          <t>Starting Portfolio Value ($)</t>
+          <t>Starting Portfolio Value (₹)</t>
         </is>
       </c>
       <c r="C10" s="103" t="n">
-        <v>50000</v>
+        <v>2000000</v>
       </c>
       <c r="D10" s="98" t="inlineStr">
         <is>
@@ -4139,11 +4139,11 @@
     <row r="11" ht="22" customHeight="1">
       <c r="B11" s="96" t="inlineStr">
         <is>
-          <t>Monthly Contribution ($)</t>
+          <t>Monthly SIP / Contribution (₹)</t>
         </is>
       </c>
       <c r="C11" s="103" t="n">
-        <v>2000</v>
+        <v>50000</v>
       </c>
       <c r="D11" s="98" t="inlineStr">
         <is>
@@ -4152,7 +4152,7 @@
       </c>
       <c r="F11" s="99" t="inlineStr">
         <is>
-          <t>Monthly Income Needed (FIRE)</t>
+          <t>Monthly Income Needed at FIRE</t>
         </is>
       </c>
       <c r="G11" s="100">
@@ -4187,7 +4187,7 @@
     <row r="13" ht="22" customHeight="1">
       <c r="B13" s="96" t="inlineStr">
         <is>
-          <t>Annual Retirement Expenses ($)</t>
+          <t>Annual Retirement Expenses (₹)</t>
         </is>
       </c>
       <c r="C13" s="104">
@@ -6038,14 +6038,14 @@
     <row r="2" ht="44" customHeight="1">
       <c r="B2" s="120" t="inlineStr">
         <is>
-          <t>SAFE WITHDRAWAL RATE &amp; POST-RETIREMENT PLANNER</t>
+          <t>SAFE WITHDRAWAL RATE &amp; POST-RETIREMENT PLANNER  (₹ INR)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="24" t="inlineStr">
         <is>
-          <t>The 4% Rule: withdraw 4% of portfolio annually — historically survived 95%+ of 30-year retirements (Trinity Study)</t>
+          <t>India context: 3.5–4% SWR is conservative. With 12% equity returns &amp; 6% inflation, real return ≈ 6% — portfolios can sustain longer</t>
         </is>
       </c>
     </row>
@@ -6141,11 +6141,11 @@
     <row r="9" ht="22" customHeight="1">
       <c r="B9" s="96" t="inlineStr">
         <is>
-          <t>Inflation Rate</t>
+          <t>Inflation Rate (India CPI)</t>
         </is>
       </c>
       <c r="C9" s="101" t="n">
-        <v>0.03</v>
+        <v>0.06</v>
       </c>
       <c r="E9" s="127" t="inlineStr">
         <is>
@@ -6191,7 +6191,7 @@
         </is>
       </c>
       <c r="C11" s="101" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="E11" s="131" t="inlineStr">
         <is>
@@ -6214,7 +6214,7 @@
         </is>
       </c>
       <c r="C12" s="97" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="E12" s="133" t="inlineStr">
         <is>

</xml_diff>